<commit_message>
Se agrega cuentas por cobrar y modulo de finanzas
</commit_message>
<xml_diff>
--- a/Inventario_Repuestos.xlsx
+++ b/Inventario_Repuestos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B7D264-7F74-4F0B-AD50-1EAD7201B7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7B0B5E-8EEA-475B-B0A3-C3E2924A48B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="250">
   <si>
     <t>INVENTARIO DE REPUESTOS</t>
   </si>
@@ -288,18 +288,12 @@
     <t>Medio juego</t>
   </si>
   <si>
-    <t>Juego completo</t>
-  </si>
-  <si>
     <t>Banda 9318 Est - Mc Block FRR Delantera</t>
   </si>
   <si>
     <t xml:space="preserve">Banda 9388 Est - Mc Block NQR </t>
   </si>
   <si>
-    <t>Banda 9388 X  Mc Block NQR</t>
-  </si>
-  <si>
     <t>Banda 9133 X Mc Block Hino</t>
   </si>
   <si>
@@ -715,6 +709,81 @@
   </si>
   <si>
     <t>Retenedor transmisión NPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro de aire NPR/NQR </t>
+  </si>
+  <si>
+    <t>Filtro de aire NPR/NQR</t>
+  </si>
+  <si>
+    <t>Filtro de aire Hino 2009</t>
+  </si>
+  <si>
+    <t>Filtro de aire Hino hasta 2009</t>
+  </si>
+  <si>
+    <t>Filtro de aceite NKR/NNR</t>
+  </si>
+  <si>
+    <t>Filtro de aire NKR</t>
+  </si>
+  <si>
+    <t>Filtro de aire NKR 2024/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro de aire NKR </t>
+  </si>
+  <si>
+    <t>Kit de filtros Hino 300</t>
+  </si>
+  <si>
+    <t>Kit filtros Hino</t>
+  </si>
+  <si>
+    <t>Filtro de aire NPR Tecnifiltro</t>
+  </si>
+  <si>
+    <t>Filtro de aire NPR</t>
+  </si>
+  <si>
+    <t>Filtro acpm</t>
+  </si>
+  <si>
+    <t>Filtro de aire NKR 2004-2008</t>
+  </si>
+  <si>
+    <t>Filtro de acpm Hino 2008-2010 Ref 1345B</t>
+  </si>
+  <si>
+    <t>Filtro de aceite Hino 500 Ref 7105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro aceite Hino </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro de acpm Hino 300 Ref 13190 </t>
+  </si>
+  <si>
+    <t>Filtro acpm Hino 300</t>
+  </si>
+  <si>
+    <t>Filtro de acpm NHR Ref 7534</t>
+  </si>
+  <si>
+    <t>Filtro acpm NHR</t>
+  </si>
+  <si>
+    <t>Filtro de aceite NHR/NKR Ref 4271</t>
+  </si>
+  <si>
+    <t>Filtro de aceite NHR/NKR</t>
+  </si>
+  <si>
+    <t>Filtro de aceite NPR/NQR Ref 7041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro de aceite </t>
   </si>
 </sst>
 </file>
@@ -824,10 +893,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaInventario" displayName="TablaInventario" ref="A3:F129" totalsRowShown="0">
-  <autoFilter ref="A3:F129" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:F129">
-    <sortCondition descending="1" ref="B3:B129"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaInventario" displayName="TablaInventario" ref="A3:F135" totalsRowShown="0">
+  <autoFilter ref="A3:F135" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A103:F118">
+    <sortCondition ref="B103:B123"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Categoría"/>
@@ -1036,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1078,13 +1147,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D4" s="3">
         <v>4</v>
@@ -1093,19 +1162,19 @@
         <v>88000</v>
       </c>
       <c r="F4" s="4">
-        <f>D4*E4</f>
+        <f t="shared" ref="F4:F35" si="0">D4*E4</f>
         <v>352000</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
@@ -1114,19 +1183,19 @@
         <v>100000</v>
       </c>
       <c r="F5" s="4">
-        <f>D5*E5</f>
+        <f t="shared" si="0"/>
         <v>400000</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D6" s="3">
         <v>14</v>
@@ -1135,19 +1204,19 @@
         <v>35000</v>
       </c>
       <c r="F6" s="4">
-        <f>D6*E6</f>
+        <f t="shared" si="0"/>
         <v>490000</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D7" s="3">
         <v>38</v>
@@ -1156,7 +1225,7 @@
         <v>30000</v>
       </c>
       <c r="F7" s="4">
-        <f>D7*E7</f>
+        <f t="shared" si="0"/>
         <v>1140000</v>
       </c>
     </row>
@@ -1177,7 +1246,7 @@
         <v>195000</v>
       </c>
       <c r="F8" s="4">
-        <f>D8*E8</f>
+        <f t="shared" si="0"/>
         <v>585000</v>
       </c>
     </row>
@@ -1198,7 +1267,7 @@
         <v>155000</v>
       </c>
       <c r="F9" s="4">
-        <f>D9*E9</f>
+        <f t="shared" si="0"/>
         <v>1240000</v>
       </c>
     </row>
@@ -1219,7 +1288,7 @@
         <v>98000</v>
       </c>
       <c r="F10" s="4">
-        <f>D10*E10</f>
+        <f t="shared" si="0"/>
         <v>980000</v>
       </c>
     </row>
@@ -1240,7 +1309,7 @@
         <v>190000</v>
       </c>
       <c r="F11" s="4">
-        <f>D11*E11</f>
+        <f t="shared" si="0"/>
         <v>1900000</v>
       </c>
     </row>
@@ -1261,7 +1330,7 @@
         <v>120000</v>
       </c>
       <c r="F12" s="4">
-        <f>D12*E12</f>
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
@@ -1282,7 +1351,7 @@
         <v>85000</v>
       </c>
       <c r="F13" s="4">
-        <f>D13*E13</f>
+        <f t="shared" si="0"/>
         <v>680000</v>
       </c>
     </row>
@@ -1303,7 +1372,7 @@
         <v>165000</v>
       </c>
       <c r="F14" s="4">
-        <f>D14*E14</f>
+        <f t="shared" si="0"/>
         <v>990000</v>
       </c>
     </row>
@@ -1324,7 +1393,7 @@
         <v>146000</v>
       </c>
       <c r="F15" s="4">
-        <f>D15*E15</f>
+        <f t="shared" si="0"/>
         <v>292000</v>
       </c>
     </row>
@@ -1345,7 +1414,7 @@
         <v>130000</v>
       </c>
       <c r="F16" s="4">
-        <f>D16*E16</f>
+        <f t="shared" si="0"/>
         <v>1170000</v>
       </c>
     </row>
@@ -1366,7 +1435,7 @@
         <v>68000</v>
       </c>
       <c r="F17" s="4">
-        <f>D17*E17</f>
+        <f t="shared" si="0"/>
         <v>204000</v>
       </c>
     </row>
@@ -1387,7 +1456,7 @@
         <v>65000</v>
       </c>
       <c r="F18" s="4">
-        <f>D18*E18</f>
+        <f t="shared" si="0"/>
         <v>65000</v>
       </c>
     </row>
@@ -1408,7 +1477,7 @@
         <v>95000</v>
       </c>
       <c r="F19" s="4">
-        <f>D19*E19</f>
+        <f t="shared" si="0"/>
         <v>950000</v>
       </c>
     </row>
@@ -1429,7 +1498,7 @@
         <v>50000</v>
       </c>
       <c r="F20" s="4">
-        <f>D20*E20</f>
+        <f t="shared" si="0"/>
         <v>300000</v>
       </c>
     </row>
@@ -1450,7 +1519,7 @@
         <v>190000</v>
       </c>
       <c r="F21" s="4">
-        <f>D21*E21</f>
+        <f t="shared" si="0"/>
         <v>1330000</v>
       </c>
     </row>
@@ -1471,7 +1540,7 @@
         <v>130000</v>
       </c>
       <c r="F22" s="4">
-        <f>D22*E22</f>
+        <f t="shared" si="0"/>
         <v>130000</v>
       </c>
     </row>
@@ -1492,7 +1561,7 @@
         <v>130000</v>
       </c>
       <c r="F23" s="4">
-        <f>D23*E23</f>
+        <f t="shared" si="0"/>
         <v>1040000</v>
       </c>
     </row>
@@ -1513,7 +1582,7 @@
         <v>100000</v>
       </c>
       <c r="F24" s="4">
-        <f>D24*E24</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
     </row>
@@ -1534,7 +1603,7 @@
         <v>90000</v>
       </c>
       <c r="F25" s="4">
-        <f>D25*E25</f>
+        <f t="shared" si="0"/>
         <v>90000</v>
       </c>
     </row>
@@ -1555,7 +1624,7 @@
         <v>152000</v>
       </c>
       <c r="F26" s="4">
-        <f>D26*E26</f>
+        <f t="shared" si="0"/>
         <v>1368000</v>
       </c>
     </row>
@@ -1576,7 +1645,7 @@
         <v>135000</v>
       </c>
       <c r="F27" s="4">
-        <f>D27*E27</f>
+        <f t="shared" si="0"/>
         <v>675000</v>
       </c>
     </row>
@@ -1597,7 +1666,7 @@
         <v>115000</v>
       </c>
       <c r="F28" s="4">
-        <f>D28*E28</f>
+        <f t="shared" si="0"/>
         <v>805000</v>
       </c>
     </row>
@@ -1618,7 +1687,7 @@
         <v>110000</v>
       </c>
       <c r="F29" s="4">
-        <f>D29*E29</f>
+        <f t="shared" si="0"/>
         <v>550000</v>
       </c>
     </row>
@@ -1639,19 +1708,19 @@
         <v>85000</v>
       </c>
       <c r="F30" s="4">
-        <f>D30*E30</f>
+        <f t="shared" si="0"/>
         <v>850000</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D31" s="3">
         <v>6</v>
@@ -1660,7 +1729,7 @@
         <v>100000</v>
       </c>
       <c r="F31" s="4">
-        <f>D31*E31</f>
+        <f t="shared" si="0"/>
         <v>600000</v>
       </c>
     </row>
@@ -1681,7 +1750,7 @@
         <v>50000</v>
       </c>
       <c r="F32" s="4">
-        <f>D32*E32</f>
+        <f t="shared" si="0"/>
         <v>700000</v>
       </c>
     </row>
@@ -1690,10 +1759,10 @@
         <v>52</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D33" s="3">
         <v>27</v>
@@ -1702,7 +1771,7 @@
         <v>60000</v>
       </c>
       <c r="F33" s="4">
-        <f>D33*E33</f>
+        <f t="shared" si="0"/>
         <v>1620000</v>
       </c>
     </row>
@@ -1723,7 +1792,7 @@
         <v>24000</v>
       </c>
       <c r="F34" s="4">
-        <f>D34*E34</f>
+        <f t="shared" si="0"/>
         <v>144000</v>
       </c>
     </row>
@@ -1732,10 +1801,10 @@
         <v>52</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D35" s="3">
         <v>4</v>
@@ -1744,7 +1813,7 @@
         <v>98000</v>
       </c>
       <c r="F35" s="4">
-        <f>D35*E35</f>
+        <f t="shared" si="0"/>
         <v>392000</v>
       </c>
     </row>
@@ -1765,7 +1834,7 @@
         <v>38000</v>
       </c>
       <c r="F36" s="4">
-        <f>D36*E36</f>
+        <f t="shared" ref="F36:F67" si="1">D36*E36</f>
         <v>570000</v>
       </c>
     </row>
@@ -1786,7 +1855,7 @@
         <v>25000</v>
       </c>
       <c r="F37" s="4">
-        <f>D37*E37</f>
+        <f t="shared" si="1"/>
         <v>150000</v>
       </c>
     </row>
@@ -1807,7 +1876,7 @@
         <v>20000</v>
       </c>
       <c r="F38" s="4">
-        <f>D38*E38</f>
+        <f t="shared" si="1"/>
         <v>120000</v>
       </c>
     </row>
@@ -1816,10 +1885,10 @@
         <v>52</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D39" s="3">
         <v>3</v>
@@ -1828,7 +1897,7 @@
         <v>55000</v>
       </c>
       <c r="F39" s="4">
-        <f>D39*E39</f>
+        <f t="shared" si="1"/>
         <v>165000</v>
       </c>
     </row>
@@ -1837,10 +1906,10 @@
         <v>52</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D40" s="3">
         <v>12</v>
@@ -1849,7 +1918,7 @@
         <v>50000</v>
       </c>
       <c r="F40" s="4">
-        <f>D40*E40</f>
+        <f t="shared" si="1"/>
         <v>600000</v>
       </c>
     </row>
@@ -1870,7 +1939,7 @@
         <v>25000</v>
       </c>
       <c r="F41" s="4">
-        <f>D41*E41</f>
+        <f t="shared" si="1"/>
         <v>200000</v>
       </c>
     </row>
@@ -1891,7 +1960,7 @@
         <v>44000</v>
       </c>
       <c r="F42" s="4">
-        <f>D42*E42</f>
+        <f t="shared" si="1"/>
         <v>264000</v>
       </c>
     </row>
@@ -1912,7 +1981,7 @@
         <v>50000</v>
       </c>
       <c r="F43" s="4">
-        <f>D43*E43</f>
+        <f t="shared" si="1"/>
         <v>700000</v>
       </c>
     </row>
@@ -1933,7 +2002,7 @@
         <v>30000</v>
       </c>
       <c r="F44" s="4">
-        <f>D44*E44</f>
+        <f t="shared" si="1"/>
         <v>330000</v>
       </c>
     </row>
@@ -1954,7 +2023,7 @@
         <v>32000</v>
       </c>
       <c r="F45" s="4">
-        <f>D45*E45</f>
+        <f t="shared" si="1"/>
         <v>672000</v>
       </c>
     </row>
@@ -1975,7 +2044,7 @@
         <v>28000</v>
       </c>
       <c r="F46" s="4">
-        <f>D46*E46</f>
+        <f t="shared" si="1"/>
         <v>140000</v>
       </c>
     </row>
@@ -1996,19 +2065,19 @@
         <v>35000</v>
       </c>
       <c r="F47" s="4">
-        <f>D47*E47</f>
+        <f t="shared" si="1"/>
         <v>490000</v>
       </c>
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D48" s="3">
         <v>2</v>
@@ -2017,19 +2086,19 @@
         <v>52000</v>
       </c>
       <c r="F48" s="4">
-        <f>D48*E48</f>
+        <f t="shared" si="1"/>
         <v>104000</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="D49" s="3">
         <v>1</v>
@@ -2038,19 +2107,19 @@
         <v>20000</v>
       </c>
       <c r="F49" s="4">
-        <f>D49*E49</f>
+        <f t="shared" si="1"/>
         <v>20000</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D50" s="3">
         <v>28</v>
@@ -2059,19 +2128,19 @@
         <v>15000</v>
       </c>
       <c r="F50" s="4">
-        <f>D50*E50</f>
+        <f t="shared" si="1"/>
         <v>420000</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D51" s="3">
         <v>6</v>
@@ -2080,19 +2149,19 @@
         <v>28000</v>
       </c>
       <c r="F51" s="4">
-        <f>D51*E51</f>
+        <f t="shared" si="1"/>
         <v>168000</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D52" s="3">
         <v>2</v>
@@ -2101,19 +2170,19 @@
         <v>24000</v>
       </c>
       <c r="F52" s="4">
-        <f>D52*E52</f>
+        <f t="shared" si="1"/>
         <v>48000</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D53" s="3">
         <v>1</v>
@@ -2122,19 +2191,19 @@
         <v>32000</v>
       </c>
       <c r="F53" s="4">
-        <f>D53*E53</f>
+        <f t="shared" si="1"/>
         <v>32000</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D54" s="3">
         <v>1</v>
@@ -2143,19 +2212,19 @@
         <v>28000</v>
       </c>
       <c r="F54" s="4">
-        <f>D54*E54</f>
+        <f t="shared" si="1"/>
         <v>28000</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D55" s="3">
         <v>1</v>
@@ -2164,19 +2233,19 @@
         <v>10000</v>
       </c>
       <c r="F55" s="4">
-        <f>D55*E55</f>
+        <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D56" s="3">
         <v>11</v>
@@ -2185,19 +2254,19 @@
         <v>94000</v>
       </c>
       <c r="F56" s="4">
-        <f>D56*E56</f>
+        <f t="shared" si="1"/>
         <v>1034000</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D57" s="3">
         <v>11</v>
@@ -2206,19 +2275,19 @@
         <v>55000</v>
       </c>
       <c r="F57" s="4">
-        <f>D57*E57</f>
+        <f t="shared" si="1"/>
         <v>605000</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C58" s="5" t="s">
         <v>212</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>214</v>
       </c>
       <c r="D58" s="3">
         <v>4</v>
@@ -2227,19 +2296,19 @@
         <v>210000</v>
       </c>
       <c r="F58" s="4">
-        <f>D58*E58</f>
+        <f t="shared" si="1"/>
         <v>840000</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D59" s="3">
         <v>4</v>
@@ -2248,19 +2317,19 @@
         <v>165000</v>
       </c>
       <c r="F59" s="4">
-        <f>D59*E59</f>
+        <f t="shared" si="1"/>
         <v>660000</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D60" s="3">
         <v>2</v>
@@ -2269,19 +2338,19 @@
         <v>210000</v>
       </c>
       <c r="F60" s="4">
-        <f>D60*E60</f>
+        <f t="shared" si="1"/>
         <v>420000</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D61" s="3">
         <v>2</v>
@@ -2290,19 +2359,19 @@
         <v>140000</v>
       </c>
       <c r="F61" s="4">
-        <f>D61*E61</f>
+        <f t="shared" si="1"/>
         <v>280000</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C62" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="D62" s="3">
         <v>4</v>
@@ -2311,19 +2380,19 @@
         <v>580000</v>
       </c>
       <c r="F62" s="4">
-        <f>D62*E62</f>
+        <f t="shared" si="1"/>
         <v>2320000</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D63" s="3">
         <v>1</v>
@@ -2332,19 +2401,19 @@
         <v>290000</v>
       </c>
       <c r="F63" s="4">
-        <f>D63*E63</f>
+        <f t="shared" si="1"/>
         <v>290000</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D64" s="3">
         <v>1</v>
@@ -2353,19 +2422,19 @@
         <v>324000</v>
       </c>
       <c r="F64" s="4">
-        <f>D64*E64</f>
+        <f t="shared" si="1"/>
         <v>324000</v>
       </c>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D65" s="3">
         <v>2</v>
@@ -2374,114 +2443,124 @@
         <v>220000</v>
       </c>
       <c r="F65" s="4">
-        <f>D65*E65</f>
+        <f t="shared" si="1"/>
         <v>440000</v>
       </c>
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D66" s="3">
         <v>1</v>
       </c>
-      <c r="E66" s="4"/>
+      <c r="E66" s="4">
+        <v>300000</v>
+      </c>
       <c r="F66" s="4">
-        <f>D66*E66</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>300000</v>
       </c>
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D67" s="3">
         <v>1</v>
       </c>
-      <c r="E67" s="4"/>
+      <c r="E67" s="4">
+        <v>300000</v>
+      </c>
       <c r="F67" s="4">
-        <f>D67*E67</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>300000</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D68" s="3">
         <v>1</v>
       </c>
-      <c r="E68" s="4"/>
+      <c r="E68" s="4">
+        <v>135000</v>
+      </c>
       <c r="F68" s="4">
-        <f t="shared" ref="F68:F70" si="0">D68*E68</f>
-        <v>0</v>
+        <f t="shared" ref="F68:F70" si="2">D68*E68</f>
+        <v>135000</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D69" s="3">
         <v>1</v>
       </c>
-      <c r="E69" s="4"/>
+      <c r="E69" s="4">
+        <v>180000</v>
+      </c>
       <c r="F69" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>180000</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D70" s="3">
         <v>1</v>
       </c>
-      <c r="E70" s="4"/>
+      <c r="E70" s="4">
+        <v>170000</v>
+      </c>
       <c r="F70" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>170000</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B71" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="B71" s="5" t="s">
-        <v>186</v>
-      </c>
       <c r="C71" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D71" s="3">
         <v>1</v>
@@ -2490,19 +2569,19 @@
         <v>260000</v>
       </c>
       <c r="F71" s="4">
-        <f>D71*E71</f>
+        <f t="shared" ref="F71:F102" si="3">D71*E71</f>
         <v>260000</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D72" s="3">
         <v>2</v>
@@ -2511,19 +2590,19 @@
         <v>320000</v>
       </c>
       <c r="F72" s="4">
-        <f>D72*E72</f>
+        <f t="shared" si="3"/>
         <v>640000</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D73" s="3">
         <v>1</v>
@@ -2532,19 +2611,19 @@
         <v>410000</v>
       </c>
       <c r="F73" s="4">
-        <f>D73*E73</f>
+        <f t="shared" si="3"/>
         <v>410000</v>
       </c>
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C74" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="D74" s="3">
         <v>6</v>
@@ -2553,19 +2632,19 @@
         <v>95000</v>
       </c>
       <c r="F74" s="4">
-        <f>D74*E74</f>
+        <f t="shared" si="3"/>
         <v>570000</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D75" s="3">
         <v>38</v>
@@ -2574,19 +2653,19 @@
         <v>30000</v>
       </c>
       <c r="F75" s="4">
-        <f>D75*E75</f>
+        <f t="shared" si="3"/>
         <v>1140000</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D76" s="3">
         <v>23</v>
@@ -2595,114 +2674,124 @@
         <v>35000</v>
       </c>
       <c r="F76" s="4">
-        <f>D76*E76</f>
+        <f t="shared" si="3"/>
         <v>805000</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D77" s="3">
         <v>1</v>
       </c>
-      <c r="E77" s="4"/>
+      <c r="E77" s="4">
+        <v>20000</v>
+      </c>
       <c r="F77" s="4">
-        <f>D77*E77</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>20000</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D78" s="3">
         <v>1</v>
       </c>
-      <c r="E78" s="4"/>
+      <c r="E78" s="4">
+        <v>20000</v>
+      </c>
       <c r="F78" s="4">
-        <f>D78*E78</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>20000</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D79" s="3">
         <v>1</v>
       </c>
-      <c r="E79" s="4"/>
+      <c r="E79" s="4">
+        <v>20000</v>
+      </c>
       <c r="F79" s="4">
-        <f>D79*E79</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>20000</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D80" s="3">
         <v>2</v>
       </c>
-      <c r="E80" s="4"/>
+      <c r="E80" s="4">
+        <v>20000</v>
+      </c>
       <c r="F80" s="4">
-        <f>D80*E80</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>40000</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D81" s="3">
         <v>2</v>
       </c>
-      <c r="E81" s="4"/>
+      <c r="E81" s="4">
+        <v>20000</v>
+      </c>
       <c r="F81" s="4">
-        <f>D81*E81</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>40000</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D82" s="3">
         <v>3</v>
@@ -2711,19 +2800,19 @@
         <v>27000</v>
       </c>
       <c r="F82" s="4">
-        <f>D82*E82</f>
+        <f t="shared" si="3"/>
         <v>81000</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D83" s="3">
         <v>1</v>
@@ -2732,19 +2821,19 @@
         <v>19000</v>
       </c>
       <c r="F83" s="4">
-        <f>D83*E83</f>
+        <f t="shared" si="3"/>
         <v>19000</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D84" s="3">
         <v>21</v>
@@ -2753,19 +2842,19 @@
         <v>20000</v>
       </c>
       <c r="F84" s="4">
-        <f>D84*E84</f>
+        <f t="shared" si="3"/>
         <v>420000</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D85" s="3">
         <v>3</v>
@@ -2774,19 +2863,19 @@
         <v>65000</v>
       </c>
       <c r="F85" s="4">
-        <f>D85*E85</f>
+        <f t="shared" si="3"/>
         <v>195000</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D86" s="3">
         <v>2</v>
@@ -2795,19 +2884,19 @@
         <v>65000</v>
       </c>
       <c r="F86" s="4">
-        <f>D86*E86</f>
+        <f t="shared" si="3"/>
         <v>130000</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D87" s="3">
         <v>150</v>
@@ -2816,19 +2905,19 @@
         <v>10000</v>
       </c>
       <c r="F87" s="4">
-        <f>D87*E87</f>
+        <f t="shared" si="3"/>
         <v>1500000</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D88" s="3">
         <v>50</v>
@@ -2837,19 +2926,19 @@
         <v>10000</v>
       </c>
       <c r="F88" s="4">
-        <f>D88*E88</f>
+        <f t="shared" si="3"/>
         <v>500000</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D89" s="3">
         <v>4</v>
@@ -2858,19 +2947,19 @@
         <v>8000</v>
       </c>
       <c r="F89" s="4">
-        <f>D89*E89</f>
+        <f t="shared" si="3"/>
         <v>32000</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D90" s="3">
         <v>29</v>
@@ -2879,19 +2968,19 @@
         <v>10000</v>
       </c>
       <c r="F90" s="4">
-        <f>D90*E90</f>
+        <f t="shared" si="3"/>
         <v>290000</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C91" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="D91" s="3">
         <v>208</v>
@@ -2900,19 +2989,19 @@
         <v>8000</v>
       </c>
       <c r="F91" s="4">
-        <f>D91*E91</f>
+        <f t="shared" si="3"/>
         <v>1664000</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D92" s="3">
         <v>4</v>
@@ -2921,19 +3010,19 @@
         <v>20000</v>
       </c>
       <c r="F92" s="4">
-        <f>D92*E92</f>
+        <f t="shared" si="3"/>
         <v>80000</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D93" s="3">
         <v>1</v>
@@ -2942,19 +3031,19 @@
         <v>15000</v>
       </c>
       <c r="F93" s="4">
-        <f>D93*E93</f>
+        <f t="shared" si="3"/>
         <v>15000</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D94" s="3">
         <v>5</v>
@@ -2963,19 +3052,19 @@
         <v>15000</v>
       </c>
       <c r="F94" s="4">
-        <f>D94*E94</f>
+        <f t="shared" si="3"/>
         <v>75000</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D95" s="3">
         <v>5</v>
@@ -2984,19 +3073,19 @@
         <v>15000</v>
       </c>
       <c r="F95" s="4">
-        <f>D95*E95</f>
+        <f t="shared" si="3"/>
         <v>75000</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D96" s="3">
         <v>2</v>
@@ -3005,19 +3094,19 @@
         <v>30000</v>
       </c>
       <c r="F96" s="4">
-        <f>D96*E96</f>
+        <f t="shared" si="3"/>
         <v>60000</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D97" s="3">
         <v>6</v>
@@ -3026,19 +3115,19 @@
         <v>50000</v>
       </c>
       <c r="F97" s="4">
-        <f>D97*E97</f>
+        <f t="shared" si="3"/>
         <v>300000</v>
       </c>
     </row>
     <row r="98" spans="1:6">
       <c r="A98" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D98" s="3">
         <v>10</v>
@@ -3047,19 +3136,19 @@
         <v>45000</v>
       </c>
       <c r="F98" s="4">
-        <f>D98*E98</f>
+        <f t="shared" si="3"/>
         <v>450000</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D99" s="3">
         <v>9</v>
@@ -3068,19 +3157,19 @@
         <v>24000</v>
       </c>
       <c r="F99" s="4">
-        <f>D99*E99</f>
+        <f t="shared" si="3"/>
         <v>216000</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D100" s="3">
         <v>4</v>
@@ -3089,19 +3178,19 @@
         <v>28000</v>
       </c>
       <c r="F100" s="4">
-        <f>D100*E100</f>
+        <f t="shared" si="3"/>
         <v>112000</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B101" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C101" s="5" t="s">
         <v>133</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="D101" s="3">
         <v>5</v>
@@ -3110,19 +3199,19 @@
         <v>28000</v>
       </c>
       <c r="F101" s="4">
-        <f>D101*E101</f>
+        <f t="shared" si="3"/>
         <v>140000</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D102" s="3">
         <v>2</v>
@@ -3131,7 +3220,7 @@
         <v>45000</v>
       </c>
       <c r="F102" s="4">
-        <f>D102*E102</f>
+        <f t="shared" si="3"/>
         <v>90000</v>
       </c>
     </row>
@@ -3140,20 +3229,20 @@
         <v>82</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C103" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D103" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E103" s="4">
-        <v>140000</v>
+        <v>120000</v>
       </c>
       <c r="F103" s="4">
-        <f>D103*E103</f>
-        <v>140000</v>
+        <f t="shared" ref="F103:F118" si="4">D103*E103</f>
+        <v>240000</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3161,20 +3250,20 @@
         <v>82</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D104" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E104" s="4">
-        <v>280000</v>
+        <v>130000</v>
       </c>
       <c r="F104" s="4">
-        <f>D104*E104</f>
-        <v>560000</v>
+        <f t="shared" si="4"/>
+        <v>390000</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3182,20 +3271,20 @@
         <v>82</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D105" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E105" s="4">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="F105" s="4">
-        <f>D105*E105</f>
-        <v>260000</v>
+        <f t="shared" si="4"/>
+        <v>360000</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3203,20 +3292,20 @@
         <v>82</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C106" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D106" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E106" s="4">
-        <v>124000</v>
+        <v>110000</v>
       </c>
       <c r="F106" s="4">
-        <f>D106*E106</f>
-        <v>124000</v>
+        <f t="shared" si="4"/>
+        <v>330000</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3224,20 +3313,20 @@
         <v>82</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D107" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E107" s="4">
-        <v>124000</v>
+        <v>154000</v>
       </c>
       <c r="F107" s="4">
-        <f>D107*E107</f>
-        <v>248000</v>
+        <f t="shared" si="4"/>
+        <v>154000</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3245,20 +3334,20 @@
         <v>82</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D108" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E108" s="4">
-        <v>324000</v>
+        <v>82000</v>
       </c>
       <c r="F108" s="4">
-        <f>D108*E108</f>
-        <v>324000</v>
+        <f t="shared" si="4"/>
+        <v>410000</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3266,20 +3355,20 @@
         <v>82</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C109" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D109" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109" s="4">
-        <v>162000</v>
+        <v>82000</v>
       </c>
       <c r="F109" s="4">
-        <f>D109*E109</f>
-        <v>162000</v>
+        <f t="shared" si="4"/>
+        <v>164000</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3287,20 +3376,20 @@
         <v>82</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D110" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E110" s="4">
-        <v>280000</v>
+        <v>140000</v>
       </c>
       <c r="F110" s="4">
-        <f>D110*E110</f>
-        <v>560000</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3308,20 +3397,20 @@
         <v>82</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D111" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E111" s="4">
-        <v>280000</v>
+        <v>150000</v>
       </c>
       <c r="F111" s="4">
-        <f>D111*E111</f>
-        <v>840000</v>
+        <f t="shared" si="4"/>
+        <v>600000</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3329,20 +3418,20 @@
         <v>82</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D112" s="3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E112" s="4">
-        <v>300000</v>
+        <v>140000</v>
       </c>
       <c r="F112" s="4">
-        <f>D112*E112</f>
-        <v>600000</v>
+        <f t="shared" si="4"/>
+        <v>840000</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3350,20 +3439,20 @@
         <v>82</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C113" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D113" s="3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E113" s="4">
         <v>140000</v>
       </c>
       <c r="F113" s="4">
-        <f t="shared" ref="F113:F129" si="1">D113*E113</f>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>560000</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -3371,20 +3460,20 @@
         <v>82</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D114" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E114" s="4">
-        <v>164000</v>
+        <v>162000</v>
       </c>
       <c r="F114" s="4">
-        <f t="shared" si="1"/>
-        <v>164000</v>
+        <f t="shared" si="4"/>
+        <v>486000</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -3392,20 +3481,20 @@
         <v>82</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D115" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E115" s="4">
-        <v>164000</v>
+        <v>62000</v>
       </c>
       <c r="F115" s="4">
-        <f t="shared" si="1"/>
-        <v>328000</v>
+        <f t="shared" si="4"/>
+        <v>248000</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -3413,7 +3502,7 @@
         <v>82</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C116" s="5" t="s">
         <v>83</v>
@@ -3422,11 +3511,11 @@
         <v>1</v>
       </c>
       <c r="E116" s="4">
-        <v>82000</v>
+        <v>124000</v>
       </c>
       <c r="F116" s="4">
-        <f t="shared" si="1"/>
-        <v>82000</v>
+        <f t="shared" si="4"/>
+        <v>124000</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -3434,20 +3523,20 @@
         <v>82</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C117" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D117" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E117" s="4">
-        <v>154000</v>
+        <v>130000</v>
       </c>
       <c r="F117" s="4">
-        <f t="shared" si="1"/>
-        <v>154000</v>
+        <f t="shared" si="4"/>
+        <v>520000</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -3455,31 +3544,31 @@
         <v>82</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D118" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E118" s="4">
-        <v>220000</v>
+        <v>140000</v>
       </c>
       <c r="F118" s="4">
-        <f t="shared" si="1"/>
-        <v>220000</v>
+        <f t="shared" si="4"/>
+        <v>700000</v>
       </c>
     </row>
     <row r="119" spans="1:6">
       <c r="A119" s="5" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>83</v>
+        <v>136</v>
       </c>
       <c r="D119" s="3">
         <v>1</v>
@@ -3488,230 +3577,366 @@
         <v>110000</v>
       </c>
       <c r="F119" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="F119:F135" si="5">D119*E119</f>
         <v>110000</v>
       </c>
     </row>
     <row r="120" spans="1:6">
       <c r="A120" s="5" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>94</v>
+        <v>135</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>84</v>
+        <v>135</v>
       </c>
       <c r="D120" s="3">
         <v>1</v>
       </c>
       <c r="E120" s="4">
-        <v>240000</v>
+        <v>100000</v>
       </c>
       <c r="F120" s="4">
-        <f t="shared" si="1"/>
-        <v>240000</v>
+        <f t="shared" si="5"/>
+        <v>100000</v>
       </c>
     </row>
     <row r="121" spans="1:6">
       <c r="A121" s="5" t="s">
-        <v>82</v>
+        <v>168</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>94</v>
+        <v>175</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="D121" s="3">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E121" s="4">
-        <v>120000</v>
+        <v>30000</v>
       </c>
       <c r="F121" s="4">
-        <f t="shared" si="1"/>
-        <v>120000</v>
+        <f t="shared" si="5"/>
+        <v>660000</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" s="5" t="s">
-        <v>82</v>
+        <v>168</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>96</v>
+        <v>176</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>84</v>
+        <v>172</v>
       </c>
       <c r="D122" s="3">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E122" s="4">
-        <v>260000</v>
+        <v>28000</v>
       </c>
       <c r="F122" s="4">
-        <f t="shared" si="1"/>
-        <v>260000</v>
+        <f t="shared" si="5"/>
+        <v>392000</v>
       </c>
     </row>
     <row r="123" spans="1:6">
       <c r="A123" s="5" t="s">
-        <v>82</v>
+        <v>210</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>96</v>
+        <v>225</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>83</v>
+        <v>226</v>
       </c>
       <c r="D123" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E123" s="4">
-        <v>130000</v>
+        <v>70000</v>
       </c>
       <c r="F123" s="4">
-        <f t="shared" si="1"/>
-        <v>130000</v>
+        <f t="shared" si="5"/>
+        <v>210000</v>
       </c>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" s="5" t="s">
-        <v>82</v>
+        <v>210</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>95</v>
+        <v>227</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>84</v>
+        <v>228</v>
       </c>
       <c r="D124" s="3">
         <v>1</v>
       </c>
       <c r="E124" s="4">
-        <v>240000</v>
+        <v>75000</v>
       </c>
       <c r="F124" s="4">
-        <f t="shared" si="1"/>
-        <v>240000</v>
+        <f t="shared" si="5"/>
+        <v>75000</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="5" t="s">
-        <v>136</v>
+        <v>210</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>138</v>
+        <v>229</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>138</v>
+        <v>229</v>
       </c>
       <c r="D125" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E125" s="4">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="F125" s="4">
-        <f t="shared" si="1"/>
-        <v>110000</v>
+        <f t="shared" si="5"/>
+        <v>180000</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" s="5" t="s">
-        <v>136</v>
+        <v>210</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>137</v>
+        <v>238</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>137</v>
+        <v>230</v>
       </c>
       <c r="D126" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E126" s="4">
-        <v>100000</v>
+        <v>38000</v>
       </c>
       <c r="F126" s="4">
-        <f t="shared" si="1"/>
-        <v>100000</v>
+        <f t="shared" si="5"/>
+        <v>114000</v>
       </c>
     </row>
     <row r="127" spans="1:6">
       <c r="A127" s="5" t="s">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>177</v>
+        <v>231</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>175</v>
+        <v>232</v>
       </c>
       <c r="D127" s="3">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E127" s="4">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="F127" s="4">
-        <f t="shared" si="1"/>
-        <v>660000</v>
+        <f t="shared" si="5"/>
+        <v>100000</v>
       </c>
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="5" t="s">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>178</v>
+        <v>233</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="D128" s="3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E128" s="4">
-        <v>28000</v>
+        <v>160000</v>
       </c>
       <c r="F128" s="4">
-        <f t="shared" si="1"/>
-        <v>392000</v>
+        <f t="shared" si="5"/>
+        <v>640000</v>
       </c>
     </row>
     <row r="129" spans="1:6">
-      <c r="A129" s="5"/>
-      <c r="B129" s="5"/>
-      <c r="C129" s="5"/>
-      <c r="D129" s="3"/>
-      <c r="E129" s="4"/>
+      <c r="A129" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D129" s="3">
+        <v>2</v>
+      </c>
+      <c r="E129" s="4">
+        <v>50000</v>
+      </c>
       <c r="F129" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6">
+      <c r="A130" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D130" s="3">
+        <v>4</v>
+      </c>
+      <c r="E130" s="4">
+        <v>40000</v>
+      </c>
+      <c r="F130" s="4">
+        <f t="shared" si="5"/>
+        <v>160000</v>
       </c>
     </row>
     <row r="131" spans="1:6">
-      <c r="A131" s="11" t="s">
+      <c r="A131" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D131" s="3">
+        <v>3</v>
+      </c>
+      <c r="E131" s="4">
+        <v>50000</v>
+      </c>
+      <c r="F131" s="4">
+        <f t="shared" si="5"/>
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6">
+      <c r="A132" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D132" s="3">
+        <v>4</v>
+      </c>
+      <c r="E132" s="4">
+        <v>65000</v>
+      </c>
+      <c r="F132" s="4">
+        <f t="shared" si="5"/>
+        <v>260000</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6">
+      <c r="A133" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D133" s="3">
+        <v>8</v>
+      </c>
+      <c r="E133" s="4">
+        <v>30000</v>
+      </c>
+      <c r="F133" s="4">
+        <f t="shared" si="5"/>
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
+      <c r="A134" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D134" s="3">
+        <v>3</v>
+      </c>
+      <c r="E134" s="4">
+        <v>30000</v>
+      </c>
+      <c r="F134" s="4">
+        <f t="shared" si="5"/>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="D135" s="3">
+        <v>5</v>
+      </c>
+      <c r="E135" s="4">
+        <v>45000</v>
+      </c>
+      <c r="F135" s="4">
+        <f t="shared" si="5"/>
+        <v>225000</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
+      <c r="A137" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B131" s="11"/>
-      <c r="C131" s="11"/>
-      <c r="D131" s="8">
-        <f>SUM(D4:D129)</f>
-        <v>1127</v>
-      </c>
-      <c r="E131" s="6"/>
-      <c r="F131" s="9">
-        <f>SUM(F4:F129)</f>
-        <v>52093000</v>
+      <c r="B137" s="11"/>
+      <c r="C137" s="11"/>
+      <c r="D137" s="8">
+        <f>SUM(D4:D135)</f>
+        <v>1193</v>
+      </c>
+      <c r="E137" s="6"/>
+      <c r="F137" s="9">
+        <f>SUM(F4:F135)</f>
+        <v>56122000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A131:C131"/>
+    <mergeCell ref="A137:C137"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -3755,15 +3980,15 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <f>SUMIF(Inventario!A4:A129,A4,Inventario!D4:D129)</f>
+        <f>SUMIF(Inventario!A4:A135,A4,Inventario!D4:D135)</f>
         <v>131</v>
       </c>
       <c r="C4" s="4">
-        <f>SUMIF(Inventario!A4:A129,A4,Inventario!F4:F129)</f>
+        <f>SUMIF(Inventario!A4:A135,A4,Inventario!F4:F135)</f>
         <v>16414000</v>
       </c>
       <c r="D4">
-        <f>COUNTIF(Inventario!A4:A129,A4)</f>
+        <f>COUNTIF(Inventario!A4:A135,A4)</f>
         <v>23</v>
       </c>
     </row>
@@ -3772,15 +3997,15 @@
         <v>52</v>
       </c>
       <c r="B5">
-        <f>SUMIF(Inventario!A4:A129,A5,Inventario!D4:D129)</f>
+        <f>SUMIF(Inventario!A4:A135,A5,Inventario!D4:D135)</f>
         <v>172</v>
       </c>
       <c r="C5" s="4">
-        <f>SUMIF(Inventario!A4:A129,A5,Inventario!F4:F129)</f>
+        <f>SUMIF(Inventario!A4:A135,A5,Inventario!F4:F135)</f>
         <v>7257000</v>
       </c>
       <c r="D5">
-        <f>COUNTIF(Inventario!A4:A129,A5)</f>
+        <f>COUNTIF(Inventario!A4:A135,A5)</f>
         <v>16</v>
       </c>
     </row>

</xml_diff>